<commit_message>
AUTOMATE-34: Added new test data
</commit_message>
<xml_diff>
--- a/Assets/Excel/SmokeTestingTestData.xlsx
+++ b/Assets/Excel/SmokeTestingTestData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jseroy\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jseroy\Desktop\Timeless\Important\Automation for peer review\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2177270-5AA9-4B80-9B5E-7842AAF9BC4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B731E4C-304E-425C-81C1-105A3035B4CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51720" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{DAEDCE94-5880-43BD-9814-69B501689CEE}"/>
+    <workbookView xWindow="51480" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="5" xr2:uid="{DAEDCE94-5880-43BD-9814-69B501689CEE}"/>
   </bookViews>
   <sheets>
     <sheet name="Guardian" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1161" uniqueCount="681">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1169" uniqueCount="686">
   <si>
     <t>MRN</t>
   </si>
@@ -2084,6 +2084,21 @@
   </si>
   <si>
     <t>ui/decimal/rounding/cals</t>
+  </si>
+  <si>
+    <t>Scenario Name</t>
+  </si>
+  <si>
+    <t>Product Name</t>
+  </si>
+  <si>
+    <t>Split Powder Product to Assigned Patient</t>
+  </si>
+  <si>
+    <t>Split Powder Product to Unassigned Patient</t>
+  </si>
+  <si>
+    <t>Split Received RTU Product to Assigned Patient</t>
   </si>
 </sst>
 </file>
@@ -8517,7 +8532,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{588C229F-E3EA-442A-809A-364CBB32564D}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.7109375" bestFit="1" customWidth="1"/>
@@ -8525,9 +8540,11 @@
     <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="42.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>674</v>
       </c>
@@ -8544,8 +8561,14 @@
       <c r="F1" s="5" t="s">
         <v>677</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H1" s="5" t="s">
+        <v>681</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>676</v>
       </c>
@@ -8563,13 +8586,33 @@
         <f>1 / (29.5735296 / 100)</f>
         <v>3.3814022658965945</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H2" t="s">
+        <v>683</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>680</v>
       </c>
       <c r="B3" s="11">
         <v>0</v>
+      </c>
+      <c r="H3" t="s">
+        <v>684</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H4" t="s">
+        <v>685</v>
+      </c>
+      <c r="I4" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -8579,5 +8622,23 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D1656CBF-F2EE-4D4C-94D8-4CDF40062885}">
+          <x14:formula1>
+            <xm:f>OrderAdditives!$A:$A</xm:f>
+          </x14:formula1>
+          <xm:sqref>I2:I3</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2A04EA3F-3286-42FE-A675-C982CF07CD44}">
+          <x14:formula1>
+            <xm:f>'Order Base'!$A:$A</xm:f>
+          </x14:formula1>
+          <xm:sqref>I4</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
AUTOMATE-33: Additional column on orders tab
</commit_message>
<xml_diff>
--- a/Assets/Excel/SmokeTestingTestData.xlsx
+++ b/Assets/Excel/SmokeTestingTestData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jseroy\Desktop\Timeless\Important\Automation for peer review\Assets\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jseroy\Desktop\Timeless\Important\Automation Clone\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B731E4C-304E-425C-81C1-105A3035B4CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15A61024-FEF2-47CB-9436-FACEF172DCB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="5" xr2:uid="{DAEDCE94-5880-43BD-9814-69B501689CEE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{DAEDCE94-5880-43BD-9814-69B501689CEE}"/>
   </bookViews>
   <sheets>
     <sheet name="Guardian" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1169" uniqueCount="686">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1178" uniqueCount="692">
   <si>
     <t>MRN</t>
   </si>
@@ -2099,6 +2099,24 @@
   </si>
   <si>
     <t>Split Received RTU Product to Assigned Patient</t>
+  </si>
+  <si>
+    <t>EHM Only</t>
+  </si>
+  <si>
+    <t>EHM Only Label Note</t>
+  </si>
+  <si>
+    <t>DHM Only</t>
+  </si>
+  <si>
+    <t>DHM Only Label Note</t>
+  </si>
+  <si>
+    <t>EHM or DHM</t>
+  </si>
+  <si>
+    <t>EHM or DHM Label Note</t>
   </si>
 </sst>
 </file>
@@ -2164,7 +2182,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2196,6 +2214,8 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2810,7 +2830,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31380DA0-60E8-49BA-9807-75EAC6F400B7}">
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.28515625" bestFit="1" customWidth="1"/>
@@ -2864,9 +2884,9 @@
         <v>364</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>640</v>
+    <row r="2" spans="1:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>686</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>11</v>
@@ -2874,54 +2894,65 @@
       <c r="F2" s="4">
         <v>10</v>
       </c>
+      <c r="G2"/>
       <c r="H2" s="7" t="s">
-        <v>641</v>
-      </c>
+        <v>687</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
       <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
-      <c r="F3" s="4"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="4" t="s">
-        <v>367</v>
-      </c>
-      <c r="J3" s="4" t="str">
-        <f>IF(VLOOKUP(I3, OrderAdditives!A:B, 2, FALSE)=0, "", VLOOKUP(I3, OrderAdditives!A:B, 2, FALSE))</f>
-        <v>Enfamil Infant</v>
-      </c>
-      <c r="K3" s="9" t="b">
-        <v>0</v>
-      </c>
+      <c r="L2" s="7">
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 20*Setup!F2, IF(Setup!B2=Setup!E1, 20*Setup!E2, IF(Setup!B2=Setup!D1, 20*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>688</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="4">
+        <v>10</v>
+      </c>
+      <c r="G3"/>
+      <c r="H3" s="7" t="s">
+        <v>689</v>
+      </c>
+      <c r="I3"/>
+      <c r="J3"/>
+      <c r="K3" s="7"/>
       <c r="L3" s="7">
-        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 22*Setup!F2, IF(Setup!B2=Setup!E1, 22*Setup!E2, IF(Setup!B2=Setup!D1, 22*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="7"/>
-      <c r="B4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="4" t="s">
-        <v>499</v>
-      </c>
-      <c r="J4" s="4" t="str">
-        <f>IF(VLOOKUP(I4, OrderAdditives!A:B, 2, FALSE)=0, "", VLOOKUP(I4, OrderAdditives!A:B, 2, FALSE))</f>
-        <v>MCT Oil</v>
-      </c>
-      <c r="K4" s="9" t="b">
-        <v>0</v>
-      </c>
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 20*Setup!F2, IF(Setup!B2=Setup!E1, 20*Setup!E2, IF(Setup!B2=Setup!D1, 20*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>690</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="4">
+        <v>10</v>
+      </c>
+      <c r="G4"/>
+      <c r="H4" s="7" t="s">
+        <v>691</v>
+      </c>
+      <c r="I4"/>
+      <c r="J4"/>
+      <c r="K4" s="7"/>
       <c r="L4" s="7">
-        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 24*Setup!F2, IF(Setup!B2=Setup!E1, 24*Setup!E2, IF(Setup!B2=Setup!D1, 24*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
-        <v>24</v>
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 20*Setup!F2, IF(Setup!B2=Setup!E1, 20*Setup!E2, IF(Setup!B2=Setup!D1, 20*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>11</v>
@@ -2930,7 +2961,7 @@
         <v>10</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="K5" s="7"/>
       <c r="L5" s="7"/>
@@ -2938,6 +2969,7 @@
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
       <c r="B6" s="7"/>
+      <c r="F6" s="4"/>
       <c r="H6" s="7"/>
       <c r="I6" s="4" t="s">
         <v>367</v>
@@ -2966,15 +2998,16 @@
         <v>MCT Oil</v>
       </c>
       <c r="K7" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L7" s="7">
-        <v>0.2</v>
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 24*Setup!F2, IF(Setup!B2=Setup!E1, 24*Setup!E2, IF(Setup!B2=Setup!D1, 24*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>659</v>
+        <v>642</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>11</v>
@@ -2983,7 +3016,7 @@
         <v>10</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
@@ -2991,7 +3024,6 @@
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
-      <c r="F9" s="4"/>
       <c r="H9" s="7"/>
       <c r="I9" s="4" t="s">
         <v>367</v>
@@ -3020,16 +3052,15 @@
         <v>MCT Oil</v>
       </c>
       <c r="K10" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L10" s="7">
-        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 24*Setup!F2, IF(Setup!B2=Setup!E1, 24*Setup!E2, IF(Setup!B2=Setup!D1, 24*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
-        <v>24</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>11</v>
@@ -3038,7 +3069,7 @@
         <v>10</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
@@ -3046,6 +3077,7 @@
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="7"/>
       <c r="B12" s="7"/>
+      <c r="F12" s="4"/>
       <c r="H12" s="7"/>
       <c r="I12" s="4" t="s">
         <v>367</v>
@@ -3074,15 +3106,16 @@
         <v>MCT Oil</v>
       </c>
       <c r="K13" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L13" s="7">
-        <v>0.2</v>
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 24*Setup!F2, IF(Setup!B2=Setup!E1, 24*Setup!E2, IF(Setup!B2=Setup!D1, 24*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>11</v>
@@ -3091,7 +3124,7 @@
         <v>10</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="K14" s="7"/>
       <c r="L14" s="7"/>
@@ -3099,7 +3132,6 @@
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="7"/>
       <c r="B15" s="7"/>
-      <c r="F15" s="4"/>
       <c r="H15" s="7"/>
       <c r="I15" s="4" t="s">
         <v>367</v>
@@ -3128,16 +3160,15 @@
         <v>MCT Oil</v>
       </c>
       <c r="K16" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16" s="7">
-        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 24*Setup!F2, IF(Setup!B2=Setup!E1, 24*Setup!E2, IF(Setup!B2=Setup!D1, 24*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
-        <v>24</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>11</v>
@@ -3183,107 +3214,97 @@
         <v>MCT Oil</v>
       </c>
       <c r="K19" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L19" s="7">
-        <v>0.2</v>
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 24*Setup!F2, IF(Setup!B2=Setup!E1, 24*Setup!E2, IF(Setup!B2=Setup!D1, 24*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>644</v>
+        <v>662</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>648</v>
-      </c>
-      <c r="C20" t="s">
-        <v>26</v>
-      </c>
-      <c r="D20" t="str">
-        <f>IF(VLOOKUP(C20, 'Order Base'!A:B, 2, FALSE)=0, "", VLOOKUP(C20, 'Order Base'!A:B, 2, FALSE))</f>
-        <v>Enfamil Infant</v>
-      </c>
-      <c r="E20">
-        <f>VLOOKUP(C20, 'Order Base'!A:C, 3, FALSE)</f>
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F20" s="4">
         <v>10</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>646</v>
+        <v>641</v>
       </c>
       <c r="K20" s="7"/>
       <c r="L20" s="7"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
-        <v>647</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>648</v>
-      </c>
-      <c r="C21" t="s">
-        <v>26</v>
-      </c>
-      <c r="D21" t="str">
-        <f>IF(VLOOKUP(C21, 'Order Base'!A:B, 2, FALSE)=0, "", VLOOKUP(C21, 'Order Base'!A:B, 2, FALSE))</f>
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="F21" s="4"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="J21" s="4" t="str">
+        <f>IF(VLOOKUP(I21, OrderAdditives!A:B, 2, FALSE)=0, "", VLOOKUP(I21, OrderAdditives!A:B, 2, FALSE))</f>
         <v>Enfamil Infant</v>
       </c>
-      <c r="E21">
-        <f>VLOOKUP(C21, 'Order Base'!A:C, 3, FALSE)</f>
-        <v>20</v>
-      </c>
-      <c r="F21" s="4">
-        <v>10</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>649</v>
-      </c>
-      <c r="K21" s="7"/>
-      <c r="L21" s="7"/>
+      <c r="K21" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="L21" s="7">
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 22*Setup!F2, IF(Setup!B2=Setup!E1, 22*Setup!E2, IF(Setup!B2=Setup!D1, 22*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
+        <v>22</v>
+      </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
       <c r="B22" s="7"/>
       <c r="H22" s="7"/>
       <c r="I22" s="4" t="s">
-        <v>367</v>
+        <v>499</v>
       </c>
       <c r="J22" s="4" t="str">
         <f>IF(VLOOKUP(I22, OrderAdditives!A:B, 2, FALSE)=0, "", VLOOKUP(I22, OrderAdditives!A:B, 2, FALSE))</f>
+        <v>MCT Oil</v>
+      </c>
+      <c r="K22" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L22" s="7">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
+        <v>644</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>648</v>
+      </c>
+      <c r="C23" t="s">
+        <v>26</v>
+      </c>
+      <c r="D23" t="str">
+        <f>IF(VLOOKUP(C23, 'Order Base'!A:B, 2, FALSE)=0, "", VLOOKUP(C23, 'Order Base'!A:B, 2, FALSE))</f>
         <v>Enfamil Infant</v>
       </c>
-      <c r="K22" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="L22" s="7">
-        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 22*Setup!F2, IF(Setup!B2=Setup!E1, 22*Setup!E2, IF(Setup!B2=Setup!D1, 22*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="4" t="s">
-        <v>499</v>
-      </c>
-      <c r="J23" s="4" t="str">
-        <f>IF(VLOOKUP(I23, OrderAdditives!A:B, 2, FALSE)=0, "", VLOOKUP(I23, OrderAdditives!A:B, 2, FALSE))</f>
-        <v>MCT Oil</v>
-      </c>
-      <c r="K23" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="L23" s="7">
-        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 24*Setup!F2, IF(Setup!B2=Setup!E1, 24*Setup!E2, IF(Setup!B2=Setup!D1, 24*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
-        <v>24</v>
-      </c>
+      <c r="E23">
+        <f>VLOOKUP(C23, 'Order Base'!A:C, 3, FALSE)</f>
+        <v>20</v>
+      </c>
+      <c r="F23" s="4">
+        <v>10</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>646</v>
+      </c>
+      <c r="K23" s="7"/>
+      <c r="L23" s="7"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
-        <v>652</v>
+        <v>647</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>648</v>
@@ -3303,7 +3324,7 @@
         <v>10</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
       <c r="K24" s="7"/>
       <c r="L24" s="7"/>
@@ -3339,38 +3360,37 @@
         <v>MCT Oil</v>
       </c>
       <c r="K26" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L26" s="7">
-        <v>0.2</v>
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 24*Setup!F2, IF(Setup!B2=Setup!E1, 24*Setup!E2, IF(Setup!B2=Setup!D1, 24*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
+        <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>656</v>
+        <v>648</v>
       </c>
       <c r="C27" t="s">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="D27" t="str">
         <f>IF(VLOOKUP(C27, 'Order Base'!A:B, 2, FALSE)=0, "", VLOOKUP(C27, 'Order Base'!A:B, 2, FALSE))</f>
-        <v>Sim Sterile Water</v>
+        <v>Enfamil Infant</v>
       </c>
       <c r="E27">
         <f>VLOOKUP(C27, 'Order Base'!A:C, 3, FALSE)</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F27" s="4">
         <v>10</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>657</v>
-      </c>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
+        <v>653</v>
+      </c>
       <c r="K27" s="7"/>
       <c r="L27" s="7"/>
     </row>
@@ -3389,8 +3409,8 @@
         <v>0</v>
       </c>
       <c r="L28" s="7">
-        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 20*Setup!F2, IF(Setup!B2=Setup!E1, 20*Setup!E2, IF(Setup!B2=Setup!D1, 20*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
-        <v>20</v>
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 22*Setup!F2, IF(Setup!B2=Setup!E1, 22*Setup!E2, IF(Setup!B2=Setup!D1, 22*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
+        <v>22</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
@@ -3405,16 +3425,15 @@
         <v>MCT Oil</v>
       </c>
       <c r="K29" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L29" s="7">
-        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 22*Setup!F2, IF(Setup!B2=Setup!E1, 22*Setup!E2, IF(Setup!B2=Setup!D1, 22*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
-        <v>22</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B30" s="7" t="s">
         <v>656</v>
@@ -3434,8 +3453,10 @@
         <v>10</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>658</v>
-      </c>
+        <v>657</v>
+      </c>
+      <c r="I30" s="4"/>
+      <c r="J30" s="4"/>
       <c r="K30" s="7"/>
       <c r="L30" s="7"/>
     </row>
@@ -3470,14 +3491,79 @@
         <v>MCT Oil</v>
       </c>
       <c r="K32" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="L32" s="7">
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 22*Setup!F2, IF(Setup!B2=Setup!E1, 22*Setup!E2, IF(Setup!B2=Setup!D1, 22*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>655</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>656</v>
+      </c>
+      <c r="C33" t="s">
+        <v>76</v>
+      </c>
+      <c r="D33" t="str">
+        <f>IF(VLOOKUP(C33, 'Order Base'!A:B, 2, FALSE)=0, "", VLOOKUP(C33, 'Order Base'!A:B, 2, FALSE))</f>
+        <v>Sim Sterile Water</v>
+      </c>
+      <c r="E33">
+        <f>VLOOKUP(C33, 'Order Base'!A:C, 3, FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="F33" s="4">
+        <v>10</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>658</v>
+      </c>
+      <c r="K33" s="7"/>
+      <c r="L33" s="7"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A34" s="7"/>
+      <c r="B34" s="7"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="J34" s="4" t="str">
+        <f>IF(VLOOKUP(I34, OrderAdditives!A:B, 2, FALSE)=0, "", VLOOKUP(I34, OrderAdditives!A:B, 2, FALSE))</f>
+        <v>Enfamil Infant</v>
+      </c>
+      <c r="K34" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="L34" s="7">
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 20*Setup!F2, IF(Setup!B2=Setup!E1, 20*Setup!E2, IF(Setup!B2=Setup!D1, 20*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A35" s="7"/>
+      <c r="B35" s="7"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="4" t="s">
+        <v>499</v>
+      </c>
+      <c r="J35" s="4" t="str">
+        <f>IF(VLOOKUP(I35, OrderAdditives!A:B, 2, FALSE)=0, "", VLOOKUP(I35, OrderAdditives!A:B, 2, FALSE))</f>
+        <v>MCT Oil</v>
+      </c>
+      <c r="K35" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="L32" s="7">
+      <c r="L35" s="7">
         <v>0.2</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="K1 K3:K4 K6:K7 K9:K10 K12:K13 K15:K16 K18:K19 K22:K23 K25:K26 K28:K29 K31:K32">
+  <conditionalFormatting sqref="K1 K6:K7 K9:K10 K12:K13 K15:K16 K18:K19 K21:K22 K25:K26 K28:K29 K31:K32 K34:K35">
     <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
       <formula>FALSE</formula>
     </cfRule>
@@ -3494,13 +3580,13 @@
           <x14:formula1>
             <xm:f>OrderAdditives!$A:$A</xm:f>
           </x14:formula1>
-          <xm:sqref>I3:I4 I31:I32 I22:I23 I25:I29 I6:I7 I9:I10 I12:I13 I15:I16 I18:I19</xm:sqref>
+          <xm:sqref>I6:I7 I34:I35 I25:I26 I28:I32 I9:I10 I12:I13 I15:I16 I18:I19 I21:I22</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B08B8B12-B941-428A-9E58-B98C2DCC018E}">
           <x14:formula1>
             <xm:f>'Order Base'!$A:$A</xm:f>
           </x14:formula1>
-          <xm:sqref>C20:C21 C24 C30 C27</xm:sqref>
+          <xm:sqref>C23:C24 C27 C33 C30</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
AUTOMATE-33: Convert base cal column value to depend on app setting
</commit_message>
<xml_diff>
--- a/Assets/Excel/SmokeTestingTestData.xlsx
+++ b/Assets/Excel/SmokeTestingTestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jseroy\Desktop\Timeless\Important\Automation Clone\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15A61024-FEF2-47CB-9436-FACEF172DCB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56D95DC3-1CEB-4263-82F5-35D05AFC8B02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{DAEDCE94-5880-43BD-9814-69B501689CEE}"/>
   </bookViews>
@@ -2182,7 +2182,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2214,8 +2214,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2884,8 +2882,8 @@
         <v>364</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
         <v>686</v>
       </c>
       <c r="B2" s="7" t="s">
@@ -2894,20 +2892,17 @@
       <c r="F2" s="4">
         <v>10</v>
       </c>
-      <c r="G2"/>
       <c r="H2" s="7" t="s">
         <v>687</v>
       </c>
-      <c r="I2"/>
-      <c r="J2"/>
       <c r="K2" s="7"/>
       <c r="L2" s="7">
         <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 20*Setup!F2, IF(Setup!B2=Setup!E1, 20*Setup!E2, IF(Setup!B2=Setup!D1, 20*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
         <v>688</v>
       </c>
       <c r="B3" s="7" t="s">
@@ -2916,20 +2911,17 @@
       <c r="F3" s="4">
         <v>10</v>
       </c>
-      <c r="G3"/>
       <c r="H3" s="7" t="s">
         <v>689</v>
       </c>
-      <c r="I3"/>
-      <c r="J3"/>
       <c r="K3" s="7"/>
       <c r="L3" s="7">
         <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 20*Setup!F2, IF(Setup!B2=Setup!E1, 20*Setup!E2, IF(Setup!B2=Setup!D1, 20*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
         <v>690</v>
       </c>
       <c r="B4" s="7" t="s">
@@ -2938,12 +2930,9 @@
       <c r="F4" s="4">
         <v>10</v>
       </c>
-      <c r="G4"/>
       <c r="H4" s="7" t="s">
         <v>691</v>
       </c>
-      <c r="I4"/>
-      <c r="J4"/>
       <c r="K4" s="7"/>
       <c r="L4" s="7">
         <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, 20*Setup!F2, IF(Setup!B2=Setup!E1, 20*Setup!E2, IF(Setup!B2=Setup!D1, 20*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
@@ -3290,7 +3279,7 @@
         <v>Enfamil Infant</v>
       </c>
       <c r="E23">
-        <f>VLOOKUP(C23, 'Order Base'!A:C, 3, FALSE)</f>
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, VLOOKUP(C23, 'Order Base'!A:C, 3, FALSE)*Setup!F2, IF(Setup!B2=Setup!E1, VLOOKUP(C23, 'Order Base'!A:C, 3, FALSE)*Setup!E2, IF(Setup!B2=Setup!D1, VLOOKUP(C23, 'Order Base'!A:C, 3, FALSE)*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
         <v>20</v>
       </c>
       <c r="F23" s="4">
@@ -3317,7 +3306,7 @@
         <v>Enfamil Infant</v>
       </c>
       <c r="E24">
-        <f>VLOOKUP(C24, 'Order Base'!A:C, 3, FALSE)</f>
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, VLOOKUP(C24, 'Order Base'!A:C, 3, FALSE)*Setup!F2, IF(Setup!B2=Setup!E1, VLOOKUP(C24, 'Order Base'!A:C, 3, FALSE)*Setup!E2, IF(Setup!B2=Setup!D1, VLOOKUP(C24, 'Order Base'!A:C, 3, FALSE)*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
         <v>20</v>
       </c>
       <c r="F24" s="4">
@@ -3382,7 +3371,7 @@
         <v>Enfamil Infant</v>
       </c>
       <c r="E27">
-        <f>VLOOKUP(C27, 'Order Base'!A:C, 3, FALSE)</f>
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, VLOOKUP(C27, 'Order Base'!A:C, 3, FALSE)*Setup!F2, IF(Setup!B2=Setup!E1, VLOOKUP(C27, 'Order Base'!A:C, 3, FALSE)*Setup!E2, IF(Setup!B2=Setup!D1, VLOOKUP(C27, 'Order Base'!A:C, 3, FALSE)*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
         <v>20</v>
       </c>
       <c r="F27" s="4">
@@ -3446,7 +3435,7 @@
         <v>Sim Sterile Water</v>
       </c>
       <c r="E30">
-        <f>VLOOKUP(C30, 'Order Base'!A:C, 3, FALSE)</f>
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, VLOOKUP(C30, 'Order Base'!A:C, 3, FALSE)*Setup!F2, IF(Setup!B2=Setup!E1, VLOOKUP(C30, 'Order Base'!A:C, 3, FALSE)*Setup!E2, IF(Setup!B2=Setup!D1, VLOOKUP(C30, 'Order Base'!A:C, 3, FALSE)*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
         <v>0</v>
       </c>
       <c r="F30" s="4">
@@ -3513,7 +3502,7 @@
         <v>Sim Sterile Water</v>
       </c>
       <c r="E33">
-        <f>VLOOKUP(C33, 'Order Base'!A:C, 3, FALSE)</f>
+        <f>IFERROR(ROUND(IF(Setup!B2=Setup!F1, VLOOKUP(C33, 'Order Base'!A:C, 3, FALSE)*Setup!F2, IF(Setup!B2=Setup!E1, VLOOKUP(C33, 'Order Base'!A:C, 3, FALSE)*Setup!E2, IF(Setup!B2=Setup!D1, VLOOKUP(C33, 'Order Base'!A:C, 3, FALSE)*Setup!D2, 0))), IF(Setup!B2=Setup!D1, 0, Setup!B3)), 0)</f>
         <v>0</v>
       </c>
       <c r="F33" s="4">

</xml_diff>

<commit_message>
update set up background color for non editable columns
</commit_message>
<xml_diff>
--- a/Assets/Excel/SmokeTestingTestData.xlsx
+++ b/Assets/Excel/SmokeTestingTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jseroy\Desktop\Timeless\Important\Automation Clone\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56D95DC3-1CEB-4263-82F5-35D05AFC8B02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5124F267-5032-4787-9BDD-8888E62AB1B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{DAEDCE94-5880-43BD-9814-69B501689CEE}"/>
+    <workbookView xWindow="-51720" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{DAEDCE94-5880-43BD-9814-69B501689CEE}"/>
   </bookViews>
   <sheets>
     <sheet name="Guardian" sheetId="1" r:id="rId1"/>
@@ -2182,7 +2182,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2213,7 +2213,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -8620,7 +8623,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
         <v>674</v>
       </c>
       <c r="B1" s="5" t="s">
@@ -8630,13 +8633,13 @@
       <c r="D1" s="12" t="s">
         <v>678</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="6" t="s">
         <v>679</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="6" t="s">
         <v>677</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="6" t="s">
         <v>681</v>
       </c>
       <c r="I1" s="5" t="s">
@@ -8644,24 +8647,24 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="7" t="s">
         <v>676</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>678</v>
       </c>
-      <c r="D2" s="11">
+      <c r="D2" s="13">
         <v>1</v>
       </c>
-      <c r="E2" s="11">
+      <c r="E2" s="13">
         <f>1 / 29.5735296</f>
         <v>3.3814022658965943E-2</v>
       </c>
-      <c r="F2" s="11">
+      <c r="F2" s="13">
         <f>1 / (29.5735296 / 100)</f>
         <v>3.3814022658965945</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="7" t="s">
         <v>683</v>
       </c>
       <c r="I2" s="4" t="s">
@@ -8669,13 +8672,13 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="7" t="s">
         <v>680</v>
       </c>
       <c r="B3" s="11">
         <v>0</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="7" t="s">
         <v>684</v>
       </c>
       <c r="I3" s="4" t="s">
@@ -8683,7 +8686,7 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="H4" t="s">
+      <c r="H4" s="7" t="s">
         <v>685</v>
       </c>
       <c r="I4" t="s">

</xml_diff>